<commit_message>
Improve CSV/Excel cleaning: separators, number/date parsing, xlsx numeric output
- read_table/write_table: auto-detect CSV separator (;/,/tab), add --sep/--out-sep
- normalize_numbers: stop rounding to 2 decimals, resolve decimal separator by
  rightmost comma/dot, flag ambiguous "1,234"-style values as unrecognized
- normalize_dates: support "YYYY-MM-DD HH:MM:SS", count invalid dates separately
  instead of silently ignoring them
- coerce normalized numeric columns to real numbers before writing xlsx/json
- reorder clean pipeline to trim -> drop-empty -> dates -> numbers -> dedup
- split: map NaN groups to "без_значения" and suffix filename collisions
- read_table: catch any xlsx read error and exit with a clean message
- recreate sample_data/orders_export.xlsx with real Excel date/number cells
- update README (limitations, test instructions, refreshed example output)
- add pytest coverage for all of the above

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sample_data/orders_export.xlsx
+++ b/sample_data/orders_export.xlsx
@@ -16,7 +16,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -55,11 +58,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -461,15 +465,11 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>12.02.2024</t>
-        </is>
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>45334</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -481,10 +481,8 @@
           <t>Опт</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>15 000,00</t>
-        </is>
+      <c r="E2" t="n">
+        <v>15000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -493,15 +491,11 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2024-02-13</t>
-        </is>
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>45335.4375</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -513,10 +507,8 @@
           <t>Розница</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>3200.00 ₽</t>
-        </is>
+      <c r="E3" t="n">
+        <v>3200.5</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -525,15 +517,11 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>14/02/2024</t>
-        </is>
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>45336</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -545,10 +533,8 @@
           <t>Опт</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>15 000,00</t>
-        </is>
+      <c r="E4" t="n">
+        <v>15000</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -557,15 +543,11 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>14/02/2024</t>
-        </is>
+      <c r="A5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>45336</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -577,10 +559,8 @@
           <t>Опт</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>15 000,00</t>
-        </is>
+      <c r="E5" t="n">
+        <v>15000</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -589,15 +569,11 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>15.02.2024</t>
-        </is>
+      <c r="A6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>45337</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -609,10 +585,8 @@
           <t>Розница</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 890 </t>
-        </is>
+      <c r="E6" t="n">
+        <v>890</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -629,15 +603,11 @@
       <c r="F7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>2024-02-16</t>
-        </is>
+      <c r="A8" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>45338</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -649,10 +619,8 @@
           <t>Опт</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>27 400,00</t>
-        </is>
+      <c r="E8" t="n">
+        <v>27400</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>

</xml_diff>